<commit_message>
add new sript in testNG.xml
</commit_message>
<xml_diff>
--- a/testdata/Data_Resignation.xlsx
+++ b/testdata/Data_Resignation.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="41">
   <si>
     <t>First Name</t>
   </si>
@@ -179,7 +179,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -427,6 +427,111 @@
         <v>21</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="C8" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="D8" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="E8" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="F8" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="G8" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="H8" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="I8" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="J8" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="K8" t="s" s="0">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="C9" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="D9" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="E9" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="F9" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="G9" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="H9" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="I9" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="J9" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="K9" t="s" s="0">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="C10" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="D10" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="E10" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="F10" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="G10" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="H10" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="I10" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="J10" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="K10" t="s" s="0">
+        <v>40</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>